<commit_message>
docs: updated dedication file
</commit_message>
<xml_diff>
--- a/PPL - Deliverable Documents/8-PPL-dedication.xlsx
+++ b/PPL - Deliverable Documents/8-PPL-dedication.xlsx
@@ -14,14 +14,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId10" roundtripDataChecksum="YQ0NyLGv+TGMePOS1PDYY5DfVJqJfiyqLwvZSXYrSAk="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId10" roundtripDataChecksum="n3Hs9CqCbVA65PGIorzLT098FexvNh5NN0NlLjOxruQ="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
   <si>
     <t>Nombre</t>
   </si>
@@ -185,15 +185,6 @@
     <t>COMENTARIOS:</t>
   </si>
   <si>
-    <t>Debido a la mala organización que se ha tenido como equipo, 
-hemos tenido que desempeñar muchísimas más horas de la cuenta la mayoría de 
-los miembros en solucionar problemas de integración entre las distintas funcionalidades del 
-proyecto. 
-Adicionalmente, a raíz de la exigencia demandada para el pasado entregable DP, el equipo de presentaciones
-también ha echado más horas en dejar la presentación lo suficientemente completa y en cuadrar los tiempos 
-y las explicaciones de cada una de los tópicos a tratar que se deben incluir en la presentación.</t>
-  </si>
-  <si>
     <t>Comentarios sobre DP</t>
   </si>
 </sst>
@@ -329,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -388,9 +379,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
@@ -783,11 +773,11 @@
       <c r="C2" s="4">
         <v>1.0</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="E2" s="5">
         <v>1.15</v>
-      </c>
-      <c r="E2" s="4">
-        <v>1.14</v>
       </c>
       <c r="F2" s="4">
         <v>1.13</v>
@@ -806,10 +796,10 @@
       <c r="C3" s="4">
         <v>1.0</v>
       </c>
-      <c r="D3" s="4">
-        <v>1.13</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="D3" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E3" s="5">
         <v>1.0</v>
       </c>
       <c r="F3" s="4">
@@ -829,11 +819,11 @@
       <c r="C4" s="4">
         <v>1.0</v>
       </c>
-      <c r="D4" s="4">
-        <v>1.16</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0.91</v>
+      <c r="D4" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0.85</v>
       </c>
       <c r="F4" s="4">
         <v>0.6</v>
@@ -852,11 +842,11 @@
       <c r="C5" s="4">
         <v>1.0</v>
       </c>
-      <c r="D5" s="4">
-        <v>1.22</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1.14</v>
+      <c r="D5" s="5">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="5">
+        <v>1.1</v>
       </c>
       <c r="F5" s="4">
         <v>0.8</v>
@@ -875,8 +865,8 @@
       <c r="C6" s="4">
         <v>1.0</v>
       </c>
-      <c r="D6" s="4">
-        <v>1.07</v>
+      <c r="D6" s="5">
+        <v>1.05</v>
       </c>
       <c r="E6" s="4">
         <v>1.15</v>
@@ -898,11 +888,11 @@
       <c r="C7" s="6">
         <v>1.0</v>
       </c>
-      <c r="D7" s="4">
-        <v>1.16</v>
-      </c>
-      <c r="E7" s="4">
-        <v>0.66</v>
+      <c r="D7" s="5">
+        <v>0.85</v>
+      </c>
+      <c r="E7" s="5">
+        <v>0.7</v>
       </c>
       <c r="F7" s="4">
         <v>1.25</v>
@@ -921,11 +911,11 @@
       <c r="C8" s="4">
         <v>1.0</v>
       </c>
-      <c r="D8" s="4">
-        <v>1.45</v>
-      </c>
-      <c r="E8" s="4">
-        <v>1.22</v>
+      <c r="D8" s="5">
+        <v>1.25</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1.15</v>
       </c>
       <c r="F8" s="4">
         <v>1.0</v>
@@ -944,11 +934,11 @@
       <c r="C9" s="4">
         <v>1.0</v>
       </c>
-      <c r="D9" s="4">
-        <v>1.31</v>
-      </c>
-      <c r="E9" s="4">
-        <v>1.31</v>
+      <c r="D9" s="5">
+        <v>1.1</v>
+      </c>
+      <c r="E9" s="5">
+        <v>1.1</v>
       </c>
       <c r="F9" s="4">
         <v>1.03</v>
@@ -967,8 +957,8 @@
       <c r="C10" s="4">
         <v>1.0</v>
       </c>
-      <c r="D10" s="4">
-        <v>1.19</v>
+      <c r="D10" s="5">
+        <v>1.1</v>
       </c>
       <c r="E10" s="4">
         <v>1.0</v>
@@ -990,11 +980,11 @@
       <c r="C11" s="4">
         <v>1.0</v>
       </c>
-      <c r="D11" s="4">
-        <v>1.36</v>
-      </c>
-      <c r="E11" s="4">
-        <v>1.16</v>
+      <c r="D11" s="5">
+        <v>1.1</v>
+      </c>
+      <c r="E11" s="5">
+        <v>1.1</v>
       </c>
       <c r="F11" s="4">
         <v>1.17</v>
@@ -1013,11 +1003,11 @@
       <c r="C12" s="4">
         <v>1.0</v>
       </c>
-      <c r="D12" s="4">
-        <v>1.1</v>
-      </c>
-      <c r="E12" s="4">
-        <v>1.04</v>
+      <c r="D12" s="5">
+        <v>0.85</v>
+      </c>
+      <c r="E12" s="5">
+        <v>0.9</v>
       </c>
       <c r="F12" s="4">
         <v>1.13</v>
@@ -1036,8 +1026,8 @@
       <c r="C13" s="4">
         <v>1.0</v>
       </c>
-      <c r="D13" s="4">
-        <v>1.07</v>
+      <c r="D13" s="5">
+        <v>1.1</v>
       </c>
       <c r="E13" s="4">
         <v>1.0</v>
@@ -1059,11 +1049,11 @@
       <c r="C14" s="4">
         <v>1.0</v>
       </c>
-      <c r="D14" s="4">
-        <v>1.35</v>
-      </c>
-      <c r="E14" s="4">
-        <v>0.98</v>
+      <c r="D14" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1.0</v>
       </c>
       <c r="F14" s="4">
         <v>1.17</v>
@@ -1082,11 +1072,11 @@
       <c r="C15" s="4">
         <v>1.0</v>
       </c>
-      <c r="D15" s="4">
-        <v>1.41</v>
-      </c>
-      <c r="E15" s="4">
-        <v>1.33</v>
+      <c r="D15" s="5">
+        <v>1.1</v>
+      </c>
+      <c r="E15" s="5">
+        <v>1.1</v>
       </c>
       <c r="F15" s="4">
         <v>0.77</v>
@@ -1105,11 +1095,11 @@
       <c r="C16" s="4">
         <v>1.0</v>
       </c>
-      <c r="D16" s="4">
-        <v>1.22</v>
-      </c>
-      <c r="E16" s="4">
-        <v>0.9</v>
+      <c r="D16" s="5">
+        <v>1.1</v>
+      </c>
+      <c r="E16" s="5">
+        <v>0.95</v>
       </c>
       <c r="F16" s="4">
         <v>0.95</v>
@@ -1128,11 +1118,11 @@
       <c r="C17" s="4">
         <v>1.0</v>
       </c>
-      <c r="D17" s="4">
-        <v>1.3</v>
-      </c>
-      <c r="E17" s="4">
-        <v>1.16</v>
+      <c r="D17" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="E17" s="5">
+        <v>1.15</v>
       </c>
       <c r="F17" s="4">
         <v>1.0</v>
@@ -1151,11 +1141,11 @@
       <c r="C18" s="4">
         <v>1.0</v>
       </c>
-      <c r="D18" s="4">
-        <v>1.2</v>
-      </c>
-      <c r="E18" s="4">
-        <v>0.94</v>
+      <c r="D18" s="5">
+        <v>0.95</v>
+      </c>
+      <c r="E18" s="5">
+        <v>1.0</v>
       </c>
       <c r="F18" s="4">
         <v>0.95</v>
@@ -1174,8 +1164,8 @@
       <c r="C19" s="4">
         <v>1.0</v>
       </c>
-      <c r="D19" s="4">
-        <v>1.05</v>
+      <c r="D19" s="5">
+        <v>1.1</v>
       </c>
       <c r="E19" s="4">
         <v>1.05</v>
@@ -1197,11 +1187,11 @@
       <c r="C20" s="4">
         <v>1.0</v>
       </c>
-      <c r="D20" s="4">
-        <v>0.85</v>
-      </c>
-      <c r="E20" s="4">
-        <v>0.62</v>
+      <c r="D20" s="5">
+        <v>0.7</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0.55</v>
       </c>
       <c r="F20" s="4">
         <v>0.75</v>
@@ -1220,11 +1210,11 @@
       <c r="C21" s="4">
         <v>1.0</v>
       </c>
-      <c r="D21" s="4">
-        <v>1.17</v>
-      </c>
-      <c r="E21" s="4">
-        <v>1.05</v>
+      <c r="D21" s="5">
+        <v>1.1</v>
+      </c>
+      <c r="E21" s="5">
+        <v>1.0</v>
       </c>
       <c r="F21" s="4">
         <v>1.0</v>
@@ -1309,11 +1299,11 @@
       </c>
       <c r="D29" s="14">
         <f t="shared" si="1"/>
-        <v>1.196</v>
+        <v>1</v>
       </c>
       <c r="E29" s="14">
         <f t="shared" si="1"/>
-        <v>1.038</v>
+        <v>1</v>
       </c>
       <c r="F29" s="14">
         <f t="shared" si="1"/>
@@ -1334,11 +1324,11 @@
       </c>
       <c r="D30" s="14">
         <f t="shared" si="2"/>
-        <v>-0.196</v>
+        <v>0</v>
       </c>
       <c r="E30" s="14">
         <f t="shared" si="2"/>
-        <v>-0.038</v>
+        <v>0</v>
       </c>
       <c r="F30" s="14">
         <f t="shared" si="2"/>
@@ -9200,40 +9190,35 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="40.75"/>
-    <col customWidth="1" min="2" max="26" width="10.63"/>
+    <col customWidth="1" min="2" max="5" width="15.13"/>
+    <col customWidth="1" min="6" max="20" width="10.63"/>
+    <col customWidth="1" min="21" max="21" width="28.25"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="23.25" customHeight="1">
       <c r="A1" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="21" t="s">
-        <v>54</v>
-      </c>
+      <c r="B1" s="21"/>
       <c r="C1" s="22"/>
       <c r="D1" s="22"/>
       <c r="E1" s="22"/>
       <c r="F1" s="22"/>
       <c r="G1" s="22"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -10235,7 +10220,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>